<commit_message>
criado classe utils em support
</commit_message>
<xml_diff>
--- a/cypress/fixtures/dados.xlsx
+++ b/cypress/fixtures/dados.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>CENARIO</t>
   </si>
@@ -33,7 +33,7 @@
     <t>TELEFONE</t>
   </si>
   <si>
-    <t>ID1</t>
+    <t xml:space="preserve">Deve preencher o formulário com sucesso</t>
   </si>
   <si>
     <t xml:space="preserve">Ana Silva</t>
@@ -45,9 +45,6 @@
     <t>1199999-0001</t>
   </si>
   <si>
-    <t>ID2</t>
-  </si>
-  <si>
     <t xml:space="preserve">Bruno Costa</t>
   </si>
   <si>
@@ -55,9 +52,6 @@
   </si>
   <si>
     <t>1199999-0002</t>
-  </si>
-  <si>
-    <t>ID3</t>
   </si>
   <si>
     <t xml:space="preserve">Carla Souza</t>
@@ -73,7 +67,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <sz val="11.000000"/>
       <color theme="1"/>
@@ -81,21 +75,15 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="9.000000"/>
-      <color rgb="FFA31515"/>
-      <name val="Menlo"/>
+      <sz val="12.000000"/>
+      <color theme="1" tint="0"/>
+      <name val="Arial"/>
     </font>
     <font>
       <u/>
-      <sz val="9.000000"/>
-      <color theme="10"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11.000000"/>
-      <color theme="10"/>
-      <name val="Calibri"/>
+      <sz val="12.000000"/>
+      <color theme="1" tint="0"/>
+      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="3">
@@ -126,15 +114,15 @@
   </cellStyleXfs>
   <cellXfs count="6">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
-    <xf fontId="0" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFill="1"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf fontId="1" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
-    <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -634,78 +622,79 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col bestFit="1" min="2" max="2" width="11.00390625"/>
-    <col bestFit="1" min="3" max="3" width="6.00390625"/>
-    <col bestFit="1" min="4" max="4" width="23.28125"/>
-    <col bestFit="1" min="5" max="5" width="13.140625"/>
+    <col bestFit="1" min="1" max="1" style="1" width="44.07421875"/>
+    <col bestFit="1" min="2" max="2" style="1" width="13.50390625"/>
+    <col bestFit="1" min="3" max="3" style="1" width="6.00390625"/>
+    <col bestFit="1" min="4" max="4" style="1" width="28.78125"/>
+    <col bestFit="1" min="5" max="5" style="1" width="15.640625"/>
   </cols>
   <sheetData>
-    <row r="1" ht="14.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" ht="15">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" ht="14.25">
-      <c r="A2" t="s">
+    <row r="2" ht="15">
+      <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C2">
+      <c r="C2" s="1">
         <v>28</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="3" ht="14.25">
-      <c r="A3" t="s">
+    <row r="3" ht="15">
+      <c r="A3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" s="1">
+        <v>35</v>
+      </c>
+      <c r="D3" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C3">
-        <v>35</v>
-      </c>
-      <c r="D3" s="3" t="s">
+      <c r="E3" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E3" s="4" t="s">
+    </row>
+    <row r="4" ht="15">
+      <c r="A4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="4" ht="14.25">
-      <c r="A4" t="s">
+      <c r="C4" s="1">
+        <v>22</v>
+      </c>
+      <c r="D4" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B4" t="s">
+      <c r="E4" s="1" t="s">
         <v>14</v>
-      </c>
-      <c r="C4">
-        <v>22</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E4" t="s">
-        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
cria novo describe para formulario com xlsx
</commit_message>
<xml_diff>
--- a/cypress/fixtures/dados.xlsx
+++ b/cypress/fixtures/dados.xlsx
@@ -16,58 +16,175 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="54">
   <si>
     <t>CENARIO</t>
   </si>
   <si>
-    <t>NOME</t>
-  </si>
-  <si>
-    <t>IDADE</t>
+    <t>FIRST_NAME</t>
+  </si>
+  <si>
+    <t>LAST_NAME</t>
   </si>
   <si>
     <t>EMAIL</t>
   </si>
   <si>
-    <t>TELEFONE</t>
+    <t>GENDER</t>
+  </si>
+  <si>
+    <t>MOBILE</t>
+  </si>
+  <si>
+    <t>DAY_OF_BIRTH</t>
+  </si>
+  <si>
+    <t>MOUNTH_OF_BIRTH</t>
+  </si>
+  <si>
+    <t>YEAR_OF_BIRTH</t>
+  </si>
+  <si>
+    <t>SUBJECTS</t>
+  </si>
+  <si>
+    <t>HOBBIES</t>
+  </si>
+  <si>
+    <t>PICTURE</t>
+  </si>
+  <si>
+    <t>CURRENT_ADDRESS</t>
+  </si>
+  <si>
+    <t>STATE</t>
+  </si>
+  <si>
+    <t>CITY</t>
   </si>
   <si>
     <t xml:space="preserve">Deve preencher o formulário com sucesso</t>
   </si>
   <si>
-    <t xml:space="preserve">Ana Silva</t>
-  </si>
-  <si>
-    <t>ana.silva@example.com</t>
-  </si>
-  <si>
-    <t>1199999-0001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bruno Costa</t>
-  </si>
-  <si>
-    <t>bruno.costa@example.com</t>
-  </si>
-  <si>
-    <t>1199999-0002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Carla Souza</t>
-  </si>
-  <si>
-    <t>carla.souza@example.com</t>
-  </si>
-  <si>
-    <t>1199999-0003</t>
+    <t>Ana</t>
+  </si>
+  <si>
+    <t>Souza</t>
+  </si>
+  <si>
+    <t>ana.souza@email.com</t>
+  </si>
+  <si>
+    <t>Female</t>
+  </si>
+  <si>
+    <t>Maths</t>
+  </si>
+  <si>
+    <t>Sports</t>
+  </si>
+  <si>
+    <t>ana.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rua das Flores, 123</t>
+  </si>
+  <si>
+    <t>NCR</t>
+  </si>
+  <si>
+    <t>Delhi</t>
+  </si>
+  <si>
+    <t>Carlos</t>
+  </si>
+  <si>
+    <t>Pereira</t>
+  </si>
+  <si>
+    <t>carlos.p@email.com</t>
+  </si>
+  <si>
+    <t>Male</t>
+  </si>
+  <si>
+    <t>History</t>
+  </si>
+  <si>
+    <t>Reading</t>
+  </si>
+  <si>
+    <t>carlos.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Av. Brasil, 456</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Uttar Pradesh</t>
+  </si>
+  <si>
+    <t>Lucknow</t>
+  </si>
+  <si>
+    <t>Júlia</t>
+  </si>
+  <si>
+    <t>Fernandes</t>
+  </si>
+  <si>
+    <t>julia.fernandes@email.com</t>
+  </si>
+  <si>
+    <t>Other</t>
+  </si>
+  <si>
+    <t>Chemistry</t>
+  </si>
+  <si>
+    <t>Music</t>
+  </si>
+  <si>
+    <t>julia.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alameda Verde, 789</t>
+  </si>
+  <si>
+    <t>Haryana</t>
+  </si>
+  <si>
+    <t>Chandigarh</t>
+  </si>
+  <si>
+    <t>Rafael</t>
+  </si>
+  <si>
+    <t>Lima</t>
+  </si>
+  <si>
+    <t>rafael.lima@email.com</t>
+  </si>
+  <si>
+    <t>Physics</t>
+  </si>
+  <si>
+    <t>rafael.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rua do Sol, 321</t>
+  </si>
+  <si>
+    <t>Rajasthan</t>
+  </si>
+  <si>
+    <t>Noida</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3">
+  <fonts count="5">
     <font>
       <sz val="11.000000"/>
       <color theme="1"/>
@@ -80,9 +197,19 @@
       <name val="Arial"/>
     </font>
     <font>
+      <sz val="12.000000"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12.000000"/>
+      <color indexed="64"/>
+      <name val="Arial"/>
+    </font>
+    <font>
       <u/>
       <sz val="12.000000"/>
-      <color theme="1" tint="0"/>
+      <color theme="10"/>
       <name val="Arial"/>
     </font>
   </fonts>
@@ -100,7 +227,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left style="none"/>
       <right style="none"/>
@@ -108,21 +235,51 @@
       <bottom style="none"/>
       <diagonal style="none"/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal style="none"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
-    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf fontId="1" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf fontId="1" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="2" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="1" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="3" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="4" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="2" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -623,78 +780,255 @@
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col bestFit="1" min="1" max="1" style="1" width="44.07421875"/>
-    <col bestFit="1" min="2" max="2" style="1" width="13.50390625"/>
-    <col bestFit="1" min="3" max="3" style="1" width="6.00390625"/>
-    <col bestFit="1" min="4" max="4" style="1" width="28.78125"/>
-    <col bestFit="1" min="5" max="5" style="1" width="15.640625"/>
+    <col bestFit="1" min="2" max="2" style="1" width="15.2109375"/>
+    <col bestFit="1" min="3" max="3" style="1" width="14.28125"/>
+    <col bestFit="1" min="4" max="4" style="1" width="28.50390625"/>
+    <col bestFit="1" min="5" max="5" style="1" width="10.421875"/>
+    <col bestFit="1" customWidth="1" min="6" max="6" style="2" width="14.8515625"/>
+    <col bestFit="1" min="7" max="7" style="2" width="18.00390625"/>
+    <col bestFit="1" min="8" max="8" style="2" width="23.421875"/>
+    <col bestFit="1" min="9" max="9" style="2" width="19.50390625"/>
+    <col bestFit="1" min="10" max="10" style="2" width="12.57421875"/>
+    <col bestFit="1" min="11" max="11" style="2" width="10.78125"/>
+    <col bestFit="1" min="12" max="12" style="2" width="10.7109375"/>
+    <col bestFit="1" min="13" max="13" style="2" width="24.07421875"/>
+    <col bestFit="1" min="14" max="14" style="2" width="14.921875"/>
+    <col bestFit="1" min="15" max="15" style="2" width="12.640625"/>
   </cols>
   <sheetData>
     <row r="1" ht="15">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="4" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="2" ht="15">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F2" s="6">
+        <v>11987654321</v>
+      </c>
+      <c r="G2" s="6">
+        <v>12</v>
+      </c>
+      <c r="H2" s="6">
         <v>5</v>
       </c>
-      <c r="B2" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" s="1">
-        <v>28</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>8</v>
+      <c r="I2" s="6">
+        <v>2000</v>
+      </c>
+      <c r="J2" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="K2" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="L2" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="M2" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N2" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="O2" s="6" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="3" ht="15">
-      <c r="A3" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="1">
+      <c r="A3" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="F3" s="6">
+        <v>11912345678</v>
+      </c>
+      <c r="G3" s="6">
+        <v>3</v>
+      </c>
+      <c r="H3" s="6">
+        <v>11</v>
+      </c>
+      <c r="I3" s="6">
+        <v>1998</v>
+      </c>
+      <c r="J3" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="K3" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="L3" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="M3" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="N3" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="O3" s="6" t="s">
         <v>35</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="4" ht="15">
-      <c r="A4" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" s="1">
-        <v>22</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>14</v>
+      <c r="A4" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="F4" s="6">
+        <v>11955554444</v>
+      </c>
+      <c r="G4" s="6">
+        <v>25</v>
+      </c>
+      <c r="H4" s="6">
+        <v>2</v>
+      </c>
+      <c r="I4" s="6">
+        <v>2002</v>
+      </c>
+      <c r="J4" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="K4" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="L4" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="M4" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="N4" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="O4" s="6" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="5" ht="15">
+      <c r="A5" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="F5" s="6">
+        <v>11933332222</v>
+      </c>
+      <c r="G5" s="6">
+        <v>17</v>
+      </c>
+      <c r="H5" s="6">
+        <v>8</v>
+      </c>
+      <c r="I5" s="6">
+        <v>1999</v>
+      </c>
+      <c r="J5" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="K5" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="L5" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="M5" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="N5" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="O5" s="8" t="s">
+        <v>53</v>
       </c>
     </row>
   </sheetData>
@@ -702,6 +1036,7 @@
     <hyperlink r:id="rId1" ref="D2"/>
     <hyperlink r:id="rId2" ref="D3"/>
     <hyperlink r:id="rId3" ref="D4"/>
+    <hyperlink r:id="rId4" ref="D5"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157500000008" bottom="0.78740157500000008" header="0.31496062000000014" footer="0.31496062000000014"/>

</xml_diff>

<commit_message>
Configurado projeto para ler dados de planilha
</commit_message>
<xml_diff>
--- a/cypress/fixtures/dados.xlsx
+++ b/cypress/fixtures/dados.xlsx
@@ -16,7 +16,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="61">
+  <si>
+    <t>EXECUTAR</t>
+  </si>
   <si>
     <t>CENARIO</t>
   </si>
@@ -39,7 +42,7 @@
     <t>DAY_OF_BIRTH</t>
   </si>
   <si>
-    <t>MOUNTH_OF_BIRTH</t>
+    <t>MONTH_OF_BIRTH</t>
   </si>
   <si>
     <t>YEAR_OF_BIRTH</t>
@@ -63,6 +66,9 @@
     <t>CITY</t>
   </si>
   <si>
+    <t>Sim</t>
+  </si>
+  <si>
     <t xml:space="preserve">Deve preencher o formulário com sucesso</t>
   </si>
   <si>
@@ -78,6 +84,9 @@
     <t>Female</t>
   </si>
   <si>
+    <t>June</t>
+  </si>
+  <si>
     <t>Maths</t>
   </si>
   <si>
@@ -108,6 +117,9 @@
     <t>Male</t>
   </si>
   <si>
+    <t>December</t>
+  </si>
+  <si>
     <t>History</t>
   </si>
   <si>
@@ -126,6 +138,9 @@
     <t>Lucknow</t>
   </si>
   <si>
+    <t>Não</t>
+  </si>
+  <si>
     <t>Júlia</t>
   </si>
   <si>
@@ -138,6 +153,9 @@
     <t>Other</t>
   </si>
   <si>
+    <t>March</t>
+  </si>
+  <si>
     <t>Chemistry</t>
   </si>
   <si>
@@ -153,7 +171,7 @@
     <t>Haryana</t>
   </si>
   <si>
-    <t>Chandigarh</t>
+    <t>Karnal</t>
   </si>
   <si>
     <t>Rafael</t>
@@ -165,6 +183,9 @@
     <t>rafael.lima@email.com</t>
   </si>
   <si>
+    <t>September</t>
+  </si>
+  <si>
     <t>Physics</t>
   </si>
   <si>
@@ -177,7 +198,7 @@
     <t>Rajasthan</t>
   </si>
   <si>
-    <t>Noida</t>
+    <t>Jaipur</t>
   </si>
 </sst>
 </file>
@@ -203,7 +224,6 @@
     </font>
     <font>
       <sz val="12.000000"/>
-      <color indexed="64"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -254,12 +274,15 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="2" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf fontId="1" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -275,6 +298,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf fontId="4" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="3" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf fontId="2" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -779,264 +805,280 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col bestFit="1" min="1" max="1" style="1" width="44.07421875"/>
-    <col bestFit="1" min="2" max="2" style="1" width="15.2109375"/>
-    <col bestFit="1" min="3" max="3" style="1" width="14.28125"/>
-    <col bestFit="1" min="4" max="4" style="1" width="28.50390625"/>
-    <col bestFit="1" min="5" max="5" style="1" width="10.421875"/>
-    <col bestFit="1" customWidth="1" min="6" max="6" style="2" width="14.8515625"/>
-    <col bestFit="1" min="7" max="7" style="2" width="18.00390625"/>
-    <col bestFit="1" min="8" max="8" style="2" width="23.421875"/>
-    <col bestFit="1" min="9" max="9" style="2" width="19.50390625"/>
-    <col bestFit="1" min="10" max="10" style="2" width="12.57421875"/>
-    <col bestFit="1" min="11" max="11" style="2" width="10.78125"/>
-    <col bestFit="1" min="12" max="12" style="2" width="10.7109375"/>
-    <col bestFit="1" min="13" max="13" style="2" width="24.07421875"/>
-    <col bestFit="1" min="14" max="14" style="2" width="14.921875"/>
-    <col bestFit="1" min="15" max="15" style="2" width="12.640625"/>
+    <col bestFit="1" min="1" max="1" width="13.07421875"/>
+    <col bestFit="1" min="2" max="2" style="1" width="44.07421875"/>
+    <col bestFit="1" min="3" max="3" style="1" width="15.2109375"/>
+    <col bestFit="1" min="4" max="4" style="1" width="14.28125"/>
+    <col bestFit="1" min="5" max="5" style="1" width="28.50390625"/>
+    <col bestFit="1" min="6" max="6" style="1" width="10.421875"/>
+    <col bestFit="1" customWidth="1" min="7" max="7" style="2" width="14.8515625"/>
+    <col bestFit="1" min="8" max="8" style="2" width="18.00390625"/>
+    <col bestFit="1" min="9" max="9" style="2" width="23.421875"/>
+    <col bestFit="1" min="10" max="10" style="2" width="19.50390625"/>
+    <col bestFit="1" min="11" max="11" style="2" width="12.57421875"/>
+    <col bestFit="1" min="12" max="12" style="2" width="10.78125"/>
+    <col bestFit="1" min="13" max="13" style="2" width="10.7109375"/>
+    <col bestFit="1" min="14" max="14" style="2" width="24.07421875"/>
+    <col bestFit="1" min="15" max="15" style="2" width="14.921875"/>
+    <col bestFit="1" min="16" max="16" style="2" width="12.640625"/>
   </cols>
   <sheetData>
     <row r="1" ht="15">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="J1" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="K1" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="L1" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="M1" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="N1" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="4" t="s">
+      <c r="O1" s="5" t="s">
         <v>14</v>
+      </c>
+      <c r="P1" s="5" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="2" ht="15">
-      <c r="A2" s="5" t="s">
-        <v>15</v>
+      <c r="A2" s="2" t="s">
+        <v>16</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C2" s="6" t="s">
         <v>17</v>
       </c>
+      <c r="C2" s="7" t="s">
+        <v>18</v>
+      </c>
       <c r="D2" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="E2" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="F2" s="6">
-        <v>11987654321</v>
-      </c>
-      <c r="G2" s="6">
+      <c r="E2" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="G2" s="9">
+        <v>1198765432</v>
+      </c>
+      <c r="H2" s="9">
         <v>12</v>
       </c>
-      <c r="H2" s="6">
-        <v>5</v>
-      </c>
-      <c r="I2" s="6">
+      <c r="I2" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="J2" s="9">
         <v>2000</v>
       </c>
-      <c r="J2" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="K2" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="L2" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="M2" s="6" t="s">
+      <c r="K2" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="N2" s="6" t="s">
+      <c r="L2" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="O2" s="6" t="s">
+      <c r="M2" s="7" t="s">
         <v>25</v>
+      </c>
+      <c r="N2" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="O2" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="P2" s="7" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="3" ht="15">
-      <c r="A3" s="5" t="s">
-        <v>15</v>
+      <c r="A3" s="2" t="s">
+        <v>16</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>27</v>
+        <v>17</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>29</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="F3" s="6">
-        <v>11912345678</v>
-      </c>
-      <c r="G3" s="6">
-        <v>3</v>
-      </c>
-      <c r="H3" s="6">
-        <v>11</v>
-      </c>
-      <c r="I3" s="6">
+        <v>30</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="G3" s="9">
+        <v>1191234567</v>
+      </c>
+      <c r="H3" s="9">
+        <v>10</v>
+      </c>
+      <c r="I3" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="J3" s="9">
         <v>1998</v>
       </c>
-      <c r="J3" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="K3" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="L3" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="M3" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="N3" s="6" t="s">
+      <c r="K3" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="O3" s="6" t="s">
+      <c r="L3" s="7" t="s">
         <v>35</v>
+      </c>
+      <c r="M3" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="N3" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="O3" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="P3" s="7" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="4" ht="15">
-      <c r="A4" s="5" t="s">
-        <v>15</v>
+      <c r="A4" s="2" t="s">
+        <v>40</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>37</v>
+        <v>17</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>41</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="F4" s="6">
-        <v>11955554444</v>
-      </c>
-      <c r="G4" s="6">
+        <v>42</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="G4" s="9">
+        <v>1195555444</v>
+      </c>
+      <c r="H4" s="9">
         <v>25</v>
       </c>
-      <c r="H4" s="6">
-        <v>2</v>
-      </c>
-      <c r="I4" s="6">
+      <c r="I4" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="J4" s="9">
         <v>2002</v>
       </c>
-      <c r="J4" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="K4" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="L4" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="M4" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="N4" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="O4" s="6" t="s">
-        <v>45</v>
+      <c r="K4" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="L4" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="M4" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="N4" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="O4" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="P4" s="7" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="5" ht="15">
-      <c r="A5" s="5" t="s">
-        <v>15</v>
+      <c r="A5" s="2" t="s">
+        <v>16</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>47</v>
+        <v>17</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>52</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="F5" s="6">
-        <v>11933332222</v>
-      </c>
-      <c r="G5" s="6">
+        <v>53</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="G5" s="9">
+        <v>1193333222</v>
+      </c>
+      <c r="H5" s="9">
         <v>17</v>
       </c>
-      <c r="H5" s="6">
-        <v>8</v>
-      </c>
-      <c r="I5" s="6">
+      <c r="I5" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="J5" s="9">
         <v>1999</v>
       </c>
-      <c r="J5" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="K5" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="L5" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="M5" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="N5" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="O5" s="8" t="s">
-        <v>53</v>
+      <c r="K5" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="L5" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="M5" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="N5" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="O5" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="P5" s="10" t="s">
+        <v>60</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="D2"/>
-    <hyperlink r:id="rId2" ref="D3"/>
-    <hyperlink r:id="rId3" ref="D4"/>
-    <hyperlink r:id="rId4" ref="D5"/>
+    <hyperlink r:id="rId1" ref="E2"/>
+    <hyperlink r:id="rId2" ref="E3"/>
+    <hyperlink r:id="rId3" ref="E4"/>
+    <hyperlink r:id="rId4" ref="E5"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157500000008" bottom="0.78740157500000008" header="0.31496062000000014" footer="0.31496062000000014"/>

</xml_diff>

<commit_message>
Inserido condição apra executar testes da planilha com a coluna EXECUTAR
</commit_message>
<xml_diff>
--- a/cypress/fixtures/dados.xlsx
+++ b/cypress/fixtures/dados.xlsx
@@ -105,6 +105,9 @@
     <t>Delhi</t>
   </si>
   <si>
+    <t>Não</t>
+  </si>
+  <si>
     <t>Carlos</t>
   </si>
   <si>
@@ -136,9 +139,6 @@
   </si>
   <si>
     <t>Lucknow</t>
-  </si>
-  <si>
-    <t>Não</t>
   </si>
   <si>
     <t>Júlia</t>
@@ -896,7 +896,7 @@
         <v>1198765432</v>
       </c>
       <c r="H2" s="9">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="I2" s="9" t="s">
         <v>22</v>
@@ -925,57 +925,57 @@
     </row>
     <row r="3" ht="15">
       <c r="A3" s="2" t="s">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="B3" s="6" t="s">
         <v>17</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G3" s="9">
         <v>1191234567</v>
       </c>
       <c r="H3" s="9">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="I3" s="9" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="J3" s="9">
         <v>1998</v>
       </c>
       <c r="K3" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="L3" s="7" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="M3" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="N3" s="7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="O3" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P3" s="7" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4" ht="15">
       <c r="A4" s="2" t="s">
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>17</v>
@@ -1040,7 +1040,7 @@
         <v>54</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G5" s="9">
         <v>1193333222</v>

</xml_diff>